<commit_message>
Building grid: green rented, red complaint, orange تعهد بالإخلاء, colour key on top
Tenant.complaint and Contract.vacateUndertaking with audited, undoable
commands; buttons on the tenant page and unit drawer; grid filters per
colour; importer columns and header synonyms; assistant intents that open
the forms; seed examples (Michel Saab complaint, Ziad Mansour undertaking).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/seed/cedar-residence.xlsx
+++ b/public/seed/cedar-residence.xlsx
@@ -566,7 +566,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R5"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -661,16 +661,16 @@
         <v>350</v>
       </c>
       <c r="F2" t="str">
-        <v>today-12d</v>
+        <v>today-20d</v>
       </c>
       <c r="G2" t="str">
-        <v>today-12d+30d</v>
+        <v>today-20d+30d</v>
       </c>
       <c r="H2" t="str">
         <v>paid</v>
       </c>
       <c r="I2" t="str">
-        <v>today-7d</v>
+        <v>today-8d</v>
       </c>
       <c r="J2" t="str">
         <v>yes</v>
@@ -685,7 +685,7 @@
         <v>operating</v>
       </c>
       <c r="N2" t="str">
-        <v>INV-33915</v>
+        <v>INV-57363</v>
       </c>
       <c r="O2" t="str">
         <v/>
@@ -717,16 +717,16 @@
         <v>400</v>
       </c>
       <c r="F3" t="str">
-        <v>today-52d</v>
+        <v>today-8d</v>
       </c>
       <c r="G3" t="str">
-        <v>today-52d+30d</v>
+        <v>today-8d+30d</v>
       </c>
       <c r="H3" t="str">
         <v>paid</v>
       </c>
       <c r="I3" t="str">
-        <v>today-46d</v>
+        <v>today-2d</v>
       </c>
       <c r="J3" t="str">
         <v>yes</v>
@@ -741,7 +741,7 @@
         <v>operating</v>
       </c>
       <c r="N3" t="str">
-        <v>INV-17864</v>
+        <v>INV-68745</v>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -773,16 +773,16 @@
         <v>120</v>
       </c>
       <c r="F4" t="str">
-        <v>today-95d</v>
+        <v>today-89d</v>
       </c>
       <c r="G4" t="str">
-        <v>today-95d+30d</v>
+        <v>today-89d+30d</v>
       </c>
       <c r="H4" t="str">
         <v>paid</v>
       </c>
       <c r="I4" t="str">
-        <v>today-88d</v>
+        <v>today-86d</v>
       </c>
       <c r="J4" t="str">
         <v>yes</v>
@@ -797,7 +797,7 @@
         <v>operating</v>
       </c>
       <c r="N4" t="str">
-        <v>INV-39851</v>
+        <v>INV-77921</v>
       </c>
       <c r="O4" t="str">
         <v/>
@@ -829,16 +829,16 @@
         <v>180</v>
       </c>
       <c r="F5" t="str">
-        <v>today-162d</v>
+        <v>today-98d</v>
       </c>
       <c r="G5" t="str">
-        <v>today-162d+30d</v>
+        <v>today-98d+30d</v>
       </c>
       <c r="H5" t="str">
         <v>paid</v>
       </c>
       <c r="I5" t="str">
-        <v>today-159d</v>
+        <v>today-80d</v>
       </c>
       <c r="J5" t="str">
         <v>yes</v>
@@ -853,7 +853,7 @@
         <v>operating</v>
       </c>
       <c r="N5" t="str">
-        <v>INV-46637</v>
+        <v>INV-65771</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -868,65 +868,9 @@
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>CR</v>
-      </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <v>Nakhle Electric</v>
-      </c>
-      <c r="D6" t="str">
-        <v>maintenance</v>
-      </c>
-      <c r="E6">
-        <v>200</v>
-      </c>
-      <c r="F6" t="str">
-        <v>today-174d</v>
-      </c>
-      <c r="G6" t="str">
-        <v>today-174d+30d</v>
-      </c>
-      <c r="H6" t="str">
-        <v>paid</v>
-      </c>
-      <c r="I6" t="str">
-        <v>today-163d</v>
-      </c>
-      <c r="J6" t="str">
-        <v>yes</v>
-      </c>
-      <c r="K6" t="str">
-        <v>annual</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Panel thermal inspection — Main electrical panel</v>
-      </c>
-      <c r="M6" t="str">
-        <v>operating</v>
-      </c>
-      <c r="N6" t="str">
-        <v>INV-54602</v>
-      </c>
-      <c r="O6" t="str">
-        <v/>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
-        <v>Main electrical panel</v>
-      </c>
-      <c r="R6" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1505,7 +1449,7 @@
         <v>AXA Middle East</v>
       </c>
       <c r="P2" t="str">
-        <v>AXA-283876</v>
+        <v>AXA-300619</v>
       </c>
       <c r="Q2" t="str">
         <v>today+11m</v>
@@ -1523,7 +1467,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K9"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1575,7 +1519,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>+961 76 725 502</v>
+        <v>+961 78 571 863</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -1593,7 +1537,7 @@
         <v>National ID</v>
       </c>
       <c r="G2" t="str">
-        <v>rafic-salam-id.pdf</v>
+        <v>rami-kabbani-id.pdf</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -1602,15 +1546,15 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>today-7y</v>
+        <v>today-6y</v>
       </c>
       <c r="K2" t="str">
-        <v>today+5y</v>
+        <v>today+7y</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>+961 76 725 502</v>
+        <v>+961 78 571 863</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -1628,16 +1572,16 @@
         <v>Signed contract</v>
       </c>
       <c r="G3" t="str">
-        <v>CR-102-01.pdf</v>
+        <v>CR-401-01.pdf</v>
       </c>
       <c r="H3" t="str">
-        <v>CR-102-01</v>
+        <v>CR-401-01</v>
       </c>
       <c r="I3" t="str">
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>today+219d-12m</v>
+        <v>today+132d-12m</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -1645,25 +1589,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>+961 81 151 658</v>
       </c>
       <c r="B4" t="str">
-        <v>CR</v>
+        <v/>
       </c>
       <c r="C4" t="str">
-        <v>Elevator 1</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>other</v>
+        <v>id</v>
       </c>
       <c r="E4" t="str">
-        <v>certificate</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>Elevator safety certificate</v>
+        <v>National ID</v>
       </c>
       <c r="G4" t="str">
-        <v>cr-elevator-1-certificate.pdf</v>
+        <v>nicolas-dagher-id.pdf</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -1672,45 +1616,45 @@
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>today-11m</v>
+        <v>today-8y</v>
       </c>
       <c r="K4" t="str">
-        <v>today+6m</v>
+        <v>today+40d</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>+961 81 151 658</v>
       </c>
       <c r="B5" t="str">
-        <v>CR</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>Fire alarm &amp; extinguishers</v>
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>other</v>
+        <v>contract</v>
       </c>
       <c r="E5" t="str">
-        <v>certificate</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Fire system compliance certificate</v>
+        <v>Signed contract</v>
       </c>
       <c r="G5" t="str">
-        <v>cr-fire-certificate.pdf</v>
+        <v>CR-102-01.pdf</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>CR-102-01</v>
       </c>
       <c r="I5" t="str">
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>today-10m</v>
+        <v>today+227d-12m</v>
       </c>
       <c r="K5" t="str">
-        <v>today+1m</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -1721,19 +1665,19 @@
         <v>CR</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>Elevator 1</v>
       </c>
       <c r="D6" t="str">
         <v>other</v>
       </c>
       <c r="E6" t="str">
-        <v>insurance</v>
+        <v>certificate</v>
       </c>
       <c r="F6" t="str">
-        <v>AXA Middle East building policy</v>
+        <v>Elevator safety certificate</v>
       </c>
       <c r="G6" t="str">
-        <v>cr-insurance-policy.pdf</v>
+        <v>cr-elevator-1-certificate.pdf</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -1742,10 +1686,10 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>today-8m</v>
+        <v>today-11m</v>
       </c>
       <c r="K6" t="str">
-        <v>today+11m</v>
+        <v>today+5m</v>
       </c>
     </row>
     <row r="7">
@@ -1756,36 +1700,106 @@
         <v>CR</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>Fire alarm &amp; extinguishers</v>
       </c>
       <c r="D7" t="str">
         <v>other</v>
       </c>
       <c r="E7" t="str">
+        <v>certificate</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Fire system compliance certificate</v>
+      </c>
+      <c r="G7" t="str">
+        <v>cr-fire-certificate.pdf</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v>today-10m</v>
+      </c>
+      <c r="K7" t="str">
+        <v>today+5m</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v>CR</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>other</v>
+      </c>
+      <c r="E8" t="str">
+        <v>insurance</v>
+      </c>
+      <c r="F8" t="str">
+        <v>AXA Middle East building policy</v>
+      </c>
+      <c r="G8" t="str">
+        <v>cr-insurance-policy.pdf</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v>today-8m</v>
+      </c>
+      <c r="K8" t="str">
+        <v>today+11m</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v>CR</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>other</v>
+      </c>
+      <c r="E9" t="str">
         <v>ownership</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F9" t="str">
         <v>Title deed</v>
       </c>
-      <c r="G7" t="str">
+      <c r="G9" t="str">
         <v>cr-title-deed.pdf</v>
       </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v>today-1m</v>
       </c>
-      <c r="K7" t="str">
+      <c r="K9" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1914,19 +1928,19 @@
         <v>2</v>
       </c>
       <c r="F2">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G2" t="str">
         <v>no</v>
       </c>
       <c r="H2">
-        <v>1125</v>
+        <v>1150</v>
       </c>
       <c r="I2">
-        <v>1125</v>
+        <v>1150</v>
       </c>
       <c r="J2">
-        <v>1200</v>
+        <v>1225</v>
       </c>
       <c r="K2" t="str">
         <v>good</v>
@@ -1955,19 +1969,19 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="G3" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="H3">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="I3">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="J3">
-        <v>950</v>
+        <v>1025</v>
       </c>
       <c r="K3" t="str">
         <v>good</v>
@@ -1996,19 +2010,19 @@
         <v>1</v>
       </c>
       <c r="F4">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G4" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="H4">
-        <v>825</v>
+        <v>725</v>
       </c>
       <c r="I4">
-        <v>825</v>
+        <v>725</v>
       </c>
       <c r="J4">
-        <v>850</v>
+        <v>775</v>
       </c>
       <c r="K4" t="str">
         <v>good</v>
@@ -2037,16 +2051,16 @@
         <v>2</v>
       </c>
       <c r="F5">
-        <v>174</v>
+        <v>142</v>
       </c>
       <c r="G5" t="str">
         <v>no</v>
       </c>
       <c r="H5">
-        <v>1125</v>
+        <v>1200</v>
       </c>
       <c r="I5">
-        <v>1125</v>
+        <v>1200</v>
       </c>
       <c r="J5">
         <v>1225</v>
@@ -2078,19 +2092,19 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="G6" t="str">
         <v>no</v>
       </c>
       <c r="H6">
-        <v>925</v>
+        <v>950</v>
       </c>
       <c r="I6">
-        <v>925</v>
+        <v>950</v>
       </c>
       <c r="J6">
-        <v>975</v>
+        <v>1000</v>
       </c>
       <c r="K6" t="str">
         <v>good</v>
@@ -2119,19 +2133,19 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G7" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="H7">
-        <v>800</v>
+        <v>725</v>
       </c>
       <c r="I7">
-        <v>800</v>
+        <v>725</v>
       </c>
       <c r="J7">
-        <v>825</v>
+        <v>775</v>
       </c>
       <c r="K7" t="str">
         <v>good</v>
@@ -2160,7 +2174,7 @@
         <v>2</v>
       </c>
       <c r="F8">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="G8" t="str">
         <v>no</v>
@@ -2172,7 +2186,7 @@
         <v>1225</v>
       </c>
       <c r="J8">
-        <v>1250</v>
+        <v>1325</v>
       </c>
       <c r="K8" t="str">
         <v>good</v>
@@ -2201,19 +2215,19 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="G9" t="str">
         <v>no</v>
       </c>
       <c r="H9">
-        <v>1025</v>
+        <v>950</v>
       </c>
       <c r="I9">
-        <v>1025</v>
+        <v>950</v>
       </c>
       <c r="J9">
-        <v>1100</v>
+        <v>975</v>
       </c>
       <c r="K9" t="str">
         <v>good</v>
@@ -2242,22 +2256,22 @@
         <v>1</v>
       </c>
       <c r="F10">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="G10" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="H10">
-        <v>825</v>
+        <v>850</v>
       </c>
       <c r="I10">
-        <v>825</v>
+        <v>850</v>
       </c>
       <c r="J10">
         <v>875</v>
       </c>
       <c r="K10" t="str">
-        <v>good</v>
+        <v>needs_work</v>
       </c>
       <c r="L10" t="str">
         <v/>
@@ -2283,19 +2297,19 @@
         <v>2</v>
       </c>
       <c r="F11">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="G11" t="str">
         <v>no</v>
       </c>
       <c r="H11">
+        <v>1150</v>
+      </c>
+      <c r="I11">
+        <v>1150</v>
+      </c>
+      <c r="J11">
         <v>1200</v>
-      </c>
-      <c r="I11">
-        <v>1200</v>
-      </c>
-      <c r="J11">
-        <v>1250</v>
       </c>
       <c r="K11" t="str">
         <v>good</v>
@@ -2324,7 +2338,7 @@
         <v>1</v>
       </c>
       <c r="F12">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="G12" t="str">
         <v>no</v>
@@ -2336,10 +2350,10 @@
         <v>975</v>
       </c>
       <c r="J12">
-        <v>1000</v>
+        <v>1025</v>
       </c>
       <c r="K12" t="str">
-        <v>fair</v>
+        <v>good</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -2365,10 +2379,10 @@
         <v>1</v>
       </c>
       <c r="F13">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="G13" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="H13">
         <v>800</v>
@@ -2377,7 +2391,7 @@
         <v>800</v>
       </c>
       <c r="J13">
-        <v>875</v>
+        <v>850</v>
       </c>
       <c r="K13" t="str">
         <v>good</v>
@@ -2406,19 +2420,19 @@
         <v>2</v>
       </c>
       <c r="F14">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="G14" t="str">
         <v>no</v>
       </c>
       <c r="H14">
-        <v>1150</v>
+        <v>1200</v>
       </c>
       <c r="I14">
-        <v>1150</v>
+        <v>1200</v>
       </c>
       <c r="J14">
-        <v>1225</v>
+        <v>1300</v>
       </c>
       <c r="K14" t="str">
         <v>good</v>
@@ -2447,22 +2461,22 @@
         <v>1</v>
       </c>
       <c r="F15">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G15" t="str">
         <v>no</v>
       </c>
       <c r="H15">
-        <v>1025</v>
+        <v>1050</v>
       </c>
       <c r="I15">
-        <v>1025</v>
+        <v>1050</v>
       </c>
       <c r="J15">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="K15" t="str">
-        <v>good</v>
+        <v>fair</v>
       </c>
       <c r="L15" t="str">
         <v/>
@@ -2488,19 +2502,19 @@
         <v>1</v>
       </c>
       <c r="F16">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G16" t="str">
         <v>no</v>
       </c>
       <c r="H16">
-        <v>825</v>
+        <v>875</v>
       </c>
       <c r="I16">
-        <v>825</v>
+        <v>875</v>
       </c>
       <c r="J16">
-        <v>875</v>
+        <v>900</v>
       </c>
       <c r="K16" t="str">
         <v>good</v>
@@ -2529,22 +2543,22 @@
         <v>2</v>
       </c>
       <c r="F17">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="G17" t="str">
         <v>no</v>
       </c>
       <c r="H17">
-        <v>1225</v>
+        <v>1175</v>
       </c>
       <c r="I17">
-        <v>1225</v>
+        <v>1175</v>
       </c>
       <c r="J17">
-        <v>1275</v>
+        <v>1250</v>
       </c>
       <c r="K17" t="str">
-        <v>fair</v>
+        <v>good</v>
       </c>
       <c r="L17" t="str">
         <v/>
@@ -2570,7 +2584,7 @@
         <v>1</v>
       </c>
       <c r="F18">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="G18" t="str">
         <v>no</v>
@@ -2585,7 +2599,7 @@
         <v>1100</v>
       </c>
       <c r="K18" t="str">
-        <v>good</v>
+        <v>needs_work</v>
       </c>
       <c r="L18" t="str">
         <v/>
@@ -2611,16 +2625,16 @@
         <v>1</v>
       </c>
       <c r="F19">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="G19" t="str">
         <v>no</v>
       </c>
       <c r="H19">
-        <v>900</v>
+        <v>875</v>
       </c>
       <c r="I19">
-        <v>900</v>
+        <v>875</v>
       </c>
       <c r="J19">
         <v>925</v>
@@ -2644,7 +2658,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:M15"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2657,6 +2671,8 @@
     <col min="9" max="9" width="24.83203125" customWidth="1"/>
     <col min="10" max="10" width="25.83203125" customWidth="1"/>
     <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2691,56 +2707,68 @@
         <v>emergency_contact_phone</v>
       </c>
       <c r="K1" t="str">
+        <v>complaint</v>
+      </c>
+      <c r="L1" t="str">
+        <v>complaint_date</v>
+      </c>
+      <c r="M1" t="str">
         <v>notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Naji</v>
+        <v>Nicolas</v>
       </c>
       <c r="B2" t="str">
-        <v>Assaf</v>
+        <v>Chamoun</v>
       </c>
       <c r="C2" t="str">
-        <v>+961 70 273 489</v>
+        <v>+961 76 307 197</v>
       </c>
       <c r="D2" t="str">
-        <v>naji.assaf@example.com</v>
+        <v>nicolas.chamoun@example.com</v>
       </c>
       <c r="E2" t="str">
-        <v>Lebanese</v>
+        <v>Canadian</v>
       </c>
       <c r="F2" t="str">
-        <v>national_id</v>
+        <v>passport</v>
       </c>
       <c r="G2" t="str">
-        <v>LB-7336817</v>
+        <v>RL9424165</v>
       </c>
       <c r="H2" t="str">
-        <v>Designer</v>
+        <v>Restaurant owner</v>
       </c>
       <c r="I2" t="str">
-        <v>Naji Assaf</v>
+        <v>Tala Chamoun</v>
       </c>
       <c r="J2" t="str">
-        <v>+961 70 132 763</v>
+        <v>+961 78 974 805</v>
       </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Rafic</v>
+        <v>Rami</v>
       </c>
       <c r="B3" t="str">
-        <v>Chahine</v>
+        <v>Kabbani</v>
       </c>
       <c r="C3" t="str">
-        <v>+961 76 677 875</v>
+        <v>+961 78 571 863</v>
       </c>
       <c r="D3" t="str">
-        <v>rafic.chahine@example.com</v>
+        <v>rami.kabbani@example.com</v>
       </c>
       <c r="E3" t="str">
         <v>Lebanese</v>
@@ -2749,33 +2777,39 @@
         <v>national_id</v>
       </c>
       <c r="G3" t="str">
-        <v>LB-1926075</v>
+        <v>LB-8916645</v>
       </c>
       <c r="H3" t="str">
-        <v>Teacher</v>
+        <v>Consultant</v>
       </c>
       <c r="I3" t="str">
-        <v>Sara Chahine</v>
+        <v>Nour Kabbani</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>+961 70 254 252</v>
       </c>
       <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Maria</v>
+        <v>Nour</v>
       </c>
       <c r="B4" t="str">
-        <v>Kanaan</v>
+        <v>Khalil</v>
       </c>
       <c r="C4" t="str">
-        <v>+961 81 756 543</v>
+        <v>+961 78 180 710</v>
       </c>
       <c r="D4" t="str">
-        <v>maria.kanaan@example.com</v>
+        <v>nour.khalil@example.com</v>
       </c>
       <c r="E4" t="str">
         <v>Lebanese</v>
@@ -2784,33 +2818,39 @@
         <v>national_id</v>
       </c>
       <c r="G4" t="str">
-        <v>LB-9046313</v>
+        <v>LB-8866764</v>
       </c>
       <c r="H4" t="str">
-        <v>Lawyer</v>
+        <v>Restaurant owner</v>
       </c>
       <c r="I4" t="str">
-        <v>Josiane Kanaan</v>
+        <v/>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>+961 3 815 249</v>
       </c>
       <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Michel</v>
+        <v>Sandra</v>
       </c>
       <c r="B5" t="str">
-        <v>Issa</v>
+        <v>Azar</v>
       </c>
       <c r="C5" t="str">
-        <v>+961 76 748 409</v>
+        <v>+961 71 520 870</v>
       </c>
       <c r="D5" t="str">
-        <v>michel.issa@example.com</v>
+        <v>sandra.azar@example.com</v>
       </c>
       <c r="E5" t="str">
         <v>Lebanese</v>
@@ -2819,33 +2859,39 @@
         <v>national_id</v>
       </c>
       <c r="G5" t="str">
-        <v>LB-6422706</v>
+        <v>LB-4291894</v>
       </c>
       <c r="H5" t="str">
-        <v>Software developer</v>
+        <v>Restaurant owner</v>
       </c>
       <c r="I5" t="str">
-        <v>Rola Issa</v>
+        <v>Nadine Azar</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>+961 70 592 342</v>
       </c>
       <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Salim</v>
+        <v>Tamara</v>
       </c>
       <c r="B6" t="str">
-        <v>Nasrallah</v>
+        <v>Nehme</v>
       </c>
       <c r="C6" t="str">
-        <v>+961 3 203 636</v>
+        <v>+961 70 825 714</v>
       </c>
       <c r="D6" t="str">
-        <v>salim.nasrallah@example.com</v>
+        <v>tamara.nehme@example.com</v>
       </c>
       <c r="E6" t="str">
         <v>Lebanese</v>
@@ -2854,68 +2900,80 @@
         <v>passport</v>
       </c>
       <c r="G6" t="str">
-        <v>RL6994790</v>
+        <v>RL8233238</v>
       </c>
       <c r="H6" t="str">
-        <v>Teacher</v>
+        <v>Engineer</v>
       </c>
       <c r="I6" t="str">
-        <v>Walid Nasrallah</v>
+        <v>Josiane Nehme</v>
       </c>
       <c r="J6" t="str">
-        <v>+961 70 204 524</v>
+        <v>+961 3 700 358</v>
       </c>
       <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Reem</v>
+        <v>Farah</v>
       </c>
       <c r="B7" t="str">
-        <v>Hobeika</v>
+        <v>Sinno</v>
       </c>
       <c r="C7" t="str">
-        <v>+961 81 657 709</v>
+        <v>+961 76 304 772</v>
       </c>
       <c r="D7" t="str">
-        <v>reem.hobeika@example.com</v>
+        <v>farah.sinno@example.com</v>
       </c>
       <c r="E7" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F7" t="str">
-        <v>passport</v>
+        <v>national_id</v>
       </c>
       <c r="G7" t="str">
-        <v>RL7630636</v>
+        <v>LB-6814072</v>
       </c>
       <c r="H7" t="str">
-        <v>Architect</v>
+        <v>Dentist</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>Elias Sinno</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>+961 71 872 957</v>
       </c>
       <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Rafic</v>
+        <v>Ghada</v>
       </c>
       <c r="B8" t="str">
-        <v>Salam</v>
+        <v>Tannous</v>
       </c>
       <c r="C8" t="str">
-        <v>+961 76 725 502</v>
+        <v>+961 79 310 662</v>
       </c>
       <c r="D8" t="str">
-        <v>rafic.salam@example.com</v>
+        <v>ghada.tannous@example.com</v>
       </c>
       <c r="E8" t="str">
         <v>Lebanese</v>
@@ -2924,33 +2982,39 @@
         <v>national_id</v>
       </c>
       <c r="G8" t="str">
-        <v>LB-7246100</v>
+        <v>LB-6091581</v>
       </c>
       <c r="H8" t="str">
-        <v>Accountant</v>
+        <v>Lawyer</v>
       </c>
       <c r="I8" t="str">
-        <v>Mirna Salam</v>
+        <v/>
       </c>
       <c r="J8" t="str">
-        <v>+961 79 254 849</v>
+        <v>+961 3 251 981</v>
       </c>
       <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Habib</v>
+        <v>Pascale</v>
       </c>
       <c r="B9" t="str">
-        <v>Sfeir</v>
+        <v>Azar</v>
       </c>
       <c r="C9" t="str">
-        <v>+961 70 375 586</v>
+        <v>+961 3 810 662</v>
       </c>
       <c r="D9" t="str">
-        <v>habib.sfeir@example.com</v>
+        <v>pascale.azar@example.com</v>
       </c>
       <c r="E9" t="str">
         <v>Lebanese</v>
@@ -2959,173 +3023,203 @@
         <v>national_id</v>
       </c>
       <c r="G9" t="str">
-        <v>LB-5689249</v>
+        <v>LB-5637188</v>
       </c>
       <c r="H9" t="str">
-        <v>Restaurant owner</v>
+        <v>Accountant</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>Jihad Azar</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>+961 71 252 720</v>
       </c>
       <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Jana</v>
+        <v>Nicolas</v>
       </c>
       <c r="B10" t="str">
-        <v>Sfeir</v>
+        <v>Dagher</v>
       </c>
       <c r="C10" t="str">
-        <v>+961 71 227 191</v>
+        <v>+961 81 151 658</v>
       </c>
       <c r="D10" t="str">
-        <v>jana.sfeir@example.com</v>
+        <v>nicolas.dagher@example.com</v>
       </c>
       <c r="E10" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F10" t="str">
-        <v>passport</v>
+        <v>national_id</v>
       </c>
       <c r="G10" t="str">
-        <v>RL4727899</v>
+        <v>LB-7380402</v>
       </c>
       <c r="H10" t="str">
-        <v>Teacher</v>
+        <v>Accountant</v>
       </c>
       <c r="I10" t="str">
-        <v>Rana Sfeir</v>
+        <v>Naji Dagher</v>
       </c>
       <c r="J10" t="str">
-        <v>+961 78 418 888</v>
+        <v/>
       </c>
       <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Youssef</v>
+        <v>Sandra</v>
       </c>
       <c r="B11" t="str">
-        <v>Osseiran</v>
+        <v>Chehab</v>
       </c>
       <c r="C11" t="str">
-        <v>+961 71 565 882</v>
+        <v>+961 70 483 286</v>
       </c>
       <c r="D11" t="str">
-        <v>youssef.osseiran@example.com</v>
+        <v>sandra.chehab@example.com</v>
       </c>
       <c r="E11" t="str">
-        <v>Canadian</v>
+        <v>Lebanese</v>
       </c>
       <c r="F11" t="str">
-        <v>passport</v>
+        <v>national_id</v>
       </c>
       <c r="G11" t="str">
-        <v>RL6429763</v>
+        <v>LB-4500727</v>
       </c>
       <c r="H11" t="str">
-        <v>Lawyer</v>
+        <v>Consultant</v>
       </c>
       <c r="I11" t="str">
         <v/>
       </c>
       <c r="J11" t="str">
-        <v>+961 76 363 346</v>
+        <v/>
       </c>
       <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Ibrahim</v>
+        <v>Bilal</v>
       </c>
       <c r="B12" t="str">
-        <v>Hanna</v>
+        <v>Hijazi</v>
       </c>
       <c r="C12" t="str">
-        <v>+961 3 686 354</v>
+        <v>+961 81 869 648</v>
       </c>
       <c r="D12" t="str">
-        <v>ibrahim.hanna@example.com</v>
+        <v>bilal.hijazi@example.com</v>
       </c>
       <c r="E12" t="str">
-        <v>French</v>
+        <v>Egyptian</v>
       </c>
       <c r="F12" t="str">
         <v>passport</v>
       </c>
       <c r="G12" t="str">
-        <v>RL6087612</v>
+        <v>RL5878846</v>
       </c>
       <c r="H12" t="str">
-        <v>Accountant</v>
+        <v>Pharmacist</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>Pascale Hijazi</v>
       </c>
       <c r="J12" t="str">
-        <v>+961 81 520 175</v>
+        <v/>
       </c>
       <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Walid</v>
+        <v>Paul</v>
       </c>
       <c r="B13" t="str">
-        <v>Hajj</v>
+        <v>Osseiran</v>
       </c>
       <c r="C13" t="str">
-        <v>+961 70 335 953</v>
+        <v>+961 76 788 318</v>
       </c>
       <c r="D13" t="str">
-        <v>walid.hajj@example.com</v>
+        <v>paul.osseiran@example.com</v>
       </c>
       <c r="E13" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F13" t="str">
-        <v>passport</v>
+        <v>national_id</v>
       </c>
       <c r="G13" t="str">
-        <v>RL9566406</v>
+        <v>LB-7464822</v>
       </c>
       <c r="H13" t="str">
-        <v>Software developer</v>
+        <v>Pharmacist</v>
       </c>
       <c r="I13" t="str">
-        <v>Lamia Hajj</v>
+        <v>Sara Osseiran</v>
       </c>
       <c r="J13" t="str">
-        <v>+961 3 972 945</v>
+        <v/>
       </c>
       <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Sami</v>
+        <v>Habib</v>
       </c>
       <c r="B14" t="str">
-        <v>Frem</v>
+        <v>Sfeir</v>
       </c>
       <c r="C14" t="str">
-        <v>+961 81 905 824</v>
+        <v>+961 70 923 879</v>
       </c>
       <c r="D14" t="str">
-        <v>sami.frem@example.com</v>
+        <v>habib.sfeir@example.com</v>
       </c>
       <c r="E14" t="str">
         <v>Lebanese</v>
@@ -3134,33 +3228,39 @@
         <v>national_id</v>
       </c>
       <c r="G14" t="str">
-        <v>LB-5879694</v>
+        <v>LB-9366668</v>
       </c>
       <c r="H14" t="str">
-        <v>Pharmacist</v>
+        <v>Designer</v>
       </c>
       <c r="I14" t="str">
-        <v>Samir Frem</v>
+        <v>Reem Sfeir</v>
       </c>
       <c r="J14" t="str">
-        <v>+961 76 407 322</v>
+        <v/>
       </c>
       <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Tarek</v>
+        <v>Samir</v>
       </c>
       <c r="B15" t="str">
-        <v>Sinno</v>
+        <v>Harb</v>
       </c>
       <c r="C15" t="str">
-        <v>+961 3 537 292</v>
+        <v>+961 71 664 448</v>
       </c>
       <c r="D15" t="str">
-        <v>tarek.sinno@example.com</v>
+        <v>samir.harb@example.com</v>
       </c>
       <c r="E15" t="str">
         <v>Lebanese</v>
@@ -3169,31 +3269,37 @@
         <v>national_id</v>
       </c>
       <c r="G15" t="str">
-        <v/>
+        <v>LB-4366546</v>
       </c>
       <c r="H15" t="str">
-        <v>Dentist</v>
+        <v>Engineer</v>
       </c>
       <c r="I15" t="str">
-        <v>Bassam Sinno</v>
+        <v>Layla Harb</v>
       </c>
       <c r="J15" t="str">
-        <v>+961 70 102 924</v>
+        <v/>
       </c>
       <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:W15"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -3213,8 +3319,11 @@
     <col min="16" max="16" width="18.83203125" customWidth="1"/>
     <col min="17" max="17" width="15.83203125" customWidth="1"/>
     <col min="18" max="18" width="15.83203125" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" customWidth="1"/>
-    <col min="20" max="20" width="17.83203125" customWidth="1"/>
+    <col min="19" max="19" width="27.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3273,39 +3382,48 @@
         <v>renewal_notes</v>
       </c>
       <c r="S1" t="str">
+        <v>vacate_undertaking_signed</v>
+      </c>
+      <c r="T1" t="str">
+        <v>vacate_by</v>
+      </c>
+      <c r="U1" t="str">
+        <v>vacate_notes</v>
+      </c>
+      <c r="V1" t="str">
         <v>notes</v>
       </c>
-      <c r="T1" t="str">
+      <c r="W1" t="str">
         <v>payment_pattern</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CR-101-01</v>
+        <v>CR-202-01</v>
       </c>
       <c r="B2" t="str">
         <v>CR</v>
       </c>
       <c r="C2" t="str">
-        <v>101</v>
+        <v>202</v>
       </c>
       <c r="D2" t="str">
-        <v>+961 70 273 489</v>
+        <v>+961 76 307 197</v>
       </c>
       <c r="E2" t="str">
-        <v>today+236d-12m</v>
+        <v>today+238d-12m</v>
       </c>
       <c r="F2" t="str">
-        <v>today+236d</v>
+        <v>today+238d</v>
       </c>
       <c r="G2">
-        <v>1125</v>
+        <v>950</v>
       </c>
       <c r="H2">
-        <v>1125</v>
+        <v>950</v>
       </c>
       <c r="I2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J2" t="str">
         <v>monthly</v>
@@ -3340,40 +3458,49 @@
       <c r="T2" t="str">
         <v/>
       </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CR-201-01</v>
+        <v>CR-401-01</v>
       </c>
       <c r="B3" t="str">
         <v>CR</v>
       </c>
       <c r="C3" t="str">
-        <v>201</v>
+        <v>401</v>
       </c>
       <c r="D3" t="str">
-        <v>+961 76 677 875</v>
+        <v>+961 78 571 863</v>
       </c>
       <c r="E3" t="str">
-        <v>today+75d-24m</v>
+        <v>today+132d-12m</v>
       </c>
       <c r="F3" t="str">
-        <v>today+75d</v>
+        <v>today+132d</v>
       </c>
       <c r="G3">
-        <v>1125</v>
+        <v>1150</v>
       </c>
       <c r="H3">
-        <v>1125</v>
+        <v>1150</v>
       </c>
       <c r="I3">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="J3" t="str">
         <v>monthly</v>
       </c>
       <c r="K3" t="str">
-        <v>cash</v>
+        <v>cheque</v>
       </c>
       <c r="L3" t="str">
         <v/>
@@ -3382,7 +3509,7 @@
         <v/>
       </c>
       <c r="N3" t="str">
-        <v>CPI-linked on renewal</v>
+        <v/>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -3400,36 +3527,45 @@
         <v/>
       </c>
       <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CR-301-01</v>
+        <v>CR-503-01</v>
       </c>
       <c r="B4" t="str">
         <v>CR</v>
       </c>
       <c r="C4" t="str">
-        <v>301</v>
+        <v>503</v>
       </c>
       <c r="D4" t="str">
-        <v>+961 81 756 543</v>
+        <v>+961 78 180 710</v>
       </c>
       <c r="E4" t="str">
-        <v>today+198d-24m</v>
+        <v>today+113d-12m</v>
       </c>
       <c r="F4" t="str">
-        <v>today+198d</v>
+        <v>today+113d</v>
       </c>
       <c r="G4">
-        <v>1225</v>
+        <v>875</v>
       </c>
       <c r="H4">
-        <v>1225</v>
+        <v>875</v>
       </c>
       <c r="I4">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J4" t="str">
         <v>monthly</v>
@@ -3464,40 +3600,49 @@
       <c r="T4" t="str">
         <v/>
       </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CR-401-01</v>
+        <v>CR-603-01</v>
       </c>
       <c r="B5" t="str">
         <v>CR</v>
       </c>
       <c r="C5" t="str">
-        <v>401</v>
+        <v>603</v>
       </c>
       <c r="D5" t="str">
-        <v>+961 76 748 409</v>
+        <v>+961 71 520 870</v>
       </c>
       <c r="E5" t="str">
-        <v>today+319d-12m</v>
+        <v>today+273d-12m</v>
       </c>
       <c r="F5" t="str">
-        <v>today+319d</v>
+        <v>today+273d</v>
       </c>
       <c r="G5">
-        <v>1200</v>
+        <v>875</v>
       </c>
       <c r="H5">
-        <v>1200</v>
+        <v>875</v>
       </c>
       <c r="I5">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J5" t="str">
         <v>monthly</v>
       </c>
       <c r="K5" t="str">
-        <v>bank_transfer</v>
+        <v>cheque</v>
       </c>
       <c r="L5" t="str">
         <v/>
@@ -3506,7 +3651,7 @@
         <v/>
       </c>
       <c r="N5" t="str">
-        <v>5% on renewal</v>
+        <v/>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -3524,42 +3669,51 @@
         <v/>
       </c>
       <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>CR-202-01</v>
+        <v>CR-302-01</v>
       </c>
       <c r="B6" t="str">
         <v>CR</v>
       </c>
       <c r="C6" t="str">
-        <v>202</v>
+        <v>302</v>
       </c>
       <c r="D6" t="str">
-        <v>+961 3 203 636</v>
+        <v>+961 70 825 714</v>
       </c>
       <c r="E6" t="str">
-        <v>today+136d-12m</v>
+        <v>today+232d-12m</v>
       </c>
       <c r="F6" t="str">
-        <v>today+136d</v>
+        <v>today+232d</v>
       </c>
       <c r="G6">
-        <v>925</v>
+        <v>950</v>
       </c>
       <c r="H6">
-        <v>925</v>
+        <v>950</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="J6" t="str">
         <v>monthly</v>
       </c>
       <c r="K6" t="str">
-        <v>cheque</v>
+        <v>bank_transfer</v>
       </c>
       <c r="L6" t="str">
         <v/>
@@ -3568,7 +3722,7 @@
         <v/>
       </c>
       <c r="N6" t="str">
-        <v>5% on renewal</v>
+        <v>3% on renewal</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -3586,42 +3740,51 @@
         <v/>
       </c>
       <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>CR-303-01</v>
+        <v>CR-101-01</v>
       </c>
       <c r="B7" t="str">
         <v>CR</v>
       </c>
       <c r="C7" t="str">
-        <v>303</v>
+        <v>101</v>
       </c>
       <c r="D7" t="str">
-        <v>+961 81 657 709</v>
+        <v>+961 76 304 772</v>
       </c>
       <c r="E7" t="str">
-        <v>today+201d-12m</v>
+        <v>today+202d-12m</v>
       </c>
       <c r="F7" t="str">
-        <v>today+201d</v>
+        <v>today+202d</v>
       </c>
       <c r="G7">
-        <v>825</v>
+        <v>1150</v>
       </c>
       <c r="H7">
-        <v>825</v>
+        <v>1150</v>
       </c>
       <c r="I7">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="J7" t="str">
         <v>monthly</v>
       </c>
       <c r="K7" t="str">
-        <v>cheque</v>
+        <v>cash</v>
       </c>
       <c r="L7" t="str">
         <v/>
@@ -3648,36 +3811,45 @@
         <v/>
       </c>
       <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CR-102-01</v>
+        <v>CR-601-01</v>
       </c>
       <c r="B8" t="str">
         <v>CR</v>
       </c>
       <c r="C8" t="str">
-        <v>102</v>
+        <v>601</v>
       </c>
       <c r="D8" t="str">
-        <v>+961 76 725 502</v>
+        <v>+961 79 310 662</v>
       </c>
       <c r="E8" t="str">
-        <v>today+219d-12m</v>
+        <v>today+258d-12m</v>
       </c>
       <c r="F8" t="str">
-        <v>today+219d</v>
+        <v>today+258d</v>
       </c>
       <c r="G8">
-        <v>900</v>
+        <v>1175</v>
       </c>
       <c r="H8">
-        <v>900</v>
+        <v>1175</v>
       </c>
       <c r="I8">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J8" t="str">
         <v>monthly</v>
@@ -3712,34 +3884,43 @@
       <c r="T8" t="str">
         <v/>
       </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CR-103-01</v>
+        <v>CR-203-01</v>
       </c>
       <c r="B9" t="str">
         <v>CR</v>
       </c>
       <c r="C9" t="str">
-        <v>103</v>
+        <v>203</v>
       </c>
       <c r="D9" t="str">
-        <v>+961 70 375 586</v>
+        <v>+961 3 810 662</v>
       </c>
       <c r="E9" t="str">
-        <v>today+82d-12m</v>
+        <v>today+279d-12m</v>
       </c>
       <c r="F9" t="str">
-        <v>today+82d</v>
+        <v>today+279d</v>
       </c>
       <c r="G9">
-        <v>825</v>
+        <v>725</v>
       </c>
       <c r="H9">
-        <v>825</v>
+        <v>725</v>
       </c>
       <c r="I9">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="J9" t="str">
         <v>monthly</v>
@@ -3774,40 +3955,49 @@
       <c r="T9" t="str">
         <v/>
       </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CR-302-01</v>
+        <v>CR-102-01</v>
       </c>
       <c r="B10" t="str">
         <v>CR</v>
       </c>
       <c r="C10" t="str">
-        <v>302</v>
+        <v>102</v>
       </c>
       <c r="D10" t="str">
-        <v>+961 71 227 191</v>
+        <v>+961 81 151 658</v>
       </c>
       <c r="E10" t="str">
-        <v>today+105d-24m</v>
+        <v>today+227d-12m</v>
       </c>
       <c r="F10" t="str">
-        <v>today+105d</v>
+        <v>today+227d</v>
       </c>
       <c r="G10">
-        <v>1025</v>
+        <v>1000</v>
       </c>
       <c r="H10">
-        <v>1025</v>
+        <v>1000</v>
       </c>
       <c r="I10">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="J10" t="str">
         <v>monthly</v>
       </c>
       <c r="K10" t="str">
-        <v>cheque</v>
+        <v>bank_transfer</v>
       </c>
       <c r="L10" t="str">
         <v/>
@@ -3834,36 +4024,45 @@
         <v/>
       </c>
       <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CR-601-01</v>
+        <v>CR-103-01</v>
       </c>
       <c r="B11" t="str">
         <v>CR</v>
       </c>
       <c r="C11" t="str">
-        <v>601</v>
+        <v>103</v>
       </c>
       <c r="D11" t="str">
-        <v>+961 71 565 882</v>
+        <v>+961 70 483 286</v>
       </c>
       <c r="E11" t="str">
-        <v>today+218d-24m</v>
+        <v>today+285d-12m</v>
       </c>
       <c r="F11" t="str">
-        <v>today+218d</v>
+        <v>today+285d</v>
       </c>
       <c r="G11">
-        <v>1225</v>
+        <v>725</v>
       </c>
       <c r="H11">
-        <v>1225</v>
+        <v>725</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="J11" t="str">
         <v>monthly</v>
@@ -3898,40 +4097,49 @@
       <c r="T11" t="str">
         <v/>
       </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CR-402-01</v>
+        <v>CR-502-01</v>
       </c>
       <c r="B12" t="str">
         <v>CR</v>
       </c>
       <c r="C12" t="str">
-        <v>402</v>
+        <v>502</v>
       </c>
       <c r="D12" t="str">
-        <v>+961 3 686 354</v>
+        <v>+961 81 869 648</v>
       </c>
       <c r="E12" t="str">
-        <v>today+118d-12m</v>
+        <v>today+196d-12m</v>
       </c>
       <c r="F12" t="str">
-        <v>today+118d</v>
+        <v>today+196d</v>
       </c>
       <c r="G12">
-        <v>975</v>
+        <v>1050</v>
       </c>
       <c r="H12">
-        <v>975</v>
+        <v>1050</v>
       </c>
       <c r="I12">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J12" t="str">
         <v>monthly</v>
       </c>
       <c r="K12" t="str">
-        <v>bank_transfer</v>
+        <v>cash</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -3940,7 +4148,7 @@
         <v/>
       </c>
       <c r="N12" t="str">
-        <v/>
+        <v>5% on renewal</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -3958,42 +4166,51 @@
         <v/>
       </c>
       <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CR-501-01</v>
+        <v>CR-402-01</v>
       </c>
       <c r="B13" t="str">
         <v>CR</v>
       </c>
       <c r="C13" t="str">
-        <v>501</v>
+        <v>402</v>
       </c>
       <c r="D13" t="str">
-        <v>+961 70 335 953</v>
+        <v>+961 76 788 318</v>
       </c>
       <c r="E13" t="str">
-        <v>today+254d-12m</v>
+        <v>today+194d-24m</v>
       </c>
       <c r="F13" t="str">
-        <v>today+254d</v>
+        <v>today+194d</v>
       </c>
       <c r="G13">
-        <v>1150</v>
+        <v>975</v>
       </c>
       <c r="H13">
-        <v>1150</v>
+        <v>975</v>
       </c>
       <c r="I13">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="J13" t="str">
         <v>monthly</v>
       </c>
       <c r="K13" t="str">
-        <v>cash</v>
+        <v>bank_transfer</v>
       </c>
       <c r="L13" t="str">
         <v/>
@@ -4002,7 +4219,7 @@
         <v/>
       </c>
       <c r="N13" t="str">
-        <v>CPI-linked on renewal</v>
+        <v/>
       </c>
       <c r="O13" t="str">
         <v/>
@@ -4020,36 +4237,45 @@
         <v/>
       </c>
       <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CR-502-01</v>
+        <v>CR-501-01</v>
       </c>
       <c r="B14" t="str">
         <v>CR</v>
       </c>
       <c r="C14" t="str">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D14" t="str">
-        <v>+961 81 905 824</v>
+        <v>+961 70 923 879</v>
       </c>
       <c r="E14" t="str">
-        <v>today+81d-12m</v>
+        <v>today+193d-12m</v>
       </c>
       <c r="F14" t="str">
-        <v>today+81d</v>
+        <v>today+193d</v>
       </c>
       <c r="G14">
-        <v>1025</v>
+        <v>1200</v>
       </c>
       <c r="H14">
-        <v>1025</v>
+        <v>1200</v>
       </c>
       <c r="I14">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="J14" t="str">
         <v>monthly</v>
@@ -4084,40 +4310,49 @@
       <c r="T14" t="str">
         <v/>
       </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CR-602-01</v>
+        <v>CR-301-01</v>
       </c>
       <c r="B15" t="str">
         <v>CR</v>
       </c>
       <c r="C15" t="str">
-        <v>602</v>
+        <v>301</v>
       </c>
       <c r="D15" t="str">
-        <v>+961 3 537 292</v>
+        <v>+961 71 664 448</v>
       </c>
       <c r="E15" t="str">
-        <v>today+82d-12m</v>
+        <v>today+153d-12m</v>
       </c>
       <c r="F15" t="str">
-        <v>today+82d</v>
+        <v>today+153d</v>
       </c>
       <c r="G15">
-        <v>1075</v>
+        <v>1225</v>
       </c>
       <c r="H15">
-        <v>1075</v>
+        <v>1225</v>
       </c>
       <c r="I15">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="J15" t="str">
         <v>monthly</v>
       </c>
       <c r="K15" t="str">
-        <v>cheque</v>
+        <v>cash</v>
       </c>
       <c r="L15" t="str">
         <v/>
@@ -4144,12 +4379,21 @@
         <v/>
       </c>
       <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4699,16 +4943,16 @@
         <v>3300</v>
       </c>
       <c r="G2" t="str">
-        <v>SCH-382101</v>
+        <v>SCH-257830</v>
       </c>
       <c r="H2" t="str">
-        <v>2017-09-14</v>
+        <v>2017-01-03</v>
       </c>
       <c r="I2">
         <v>48000</v>
       </c>
       <c r="J2" t="str">
-        <v>today-29m</v>
+        <v>today-18m</v>
       </c>
       <c r="K2" t="str">
         <v>Schindler Lebanon</v>
@@ -4717,7 +4961,7 @@
         <v>operational</v>
       </c>
       <c r="M2" t="str">
-        <v>today-75d</v>
+        <v>today-92d</v>
       </c>
       <c r="N2" t="str">
         <v/>
@@ -4743,19 +4987,19 @@
         <v>Perkins</v>
       </c>
       <c r="F3" t="str">
-        <v>P387</v>
+        <v>P336</v>
       </c>
       <c r="G3" t="str">
-        <v>PER-472804</v>
+        <v>PER-636630</v>
       </c>
       <c r="H3" t="str">
-        <v>2017-08-25</v>
+        <v>2017-02-19</v>
       </c>
       <c r="I3">
         <v>32000</v>
       </c>
       <c r="J3" t="str">
-        <v>today-17m</v>
+        <v>today-9m</v>
       </c>
       <c r="K3" t="str">
         <v>PowerGen Services</v>
@@ -4764,7 +5008,7 @@
         <v>operational</v>
       </c>
       <c r="M3" t="str">
-        <v>today-135d</v>
+        <v>today-35d</v>
       </c>
       <c r="N3" t="str">
         <v/>
@@ -4793,16 +5037,16 @@
         <v>CR 10</v>
       </c>
       <c r="G4" t="str">
-        <v>GRU-159495</v>
+        <v>GRU-204229</v>
       </c>
       <c r="H4" t="str">
-        <v>2017-10-05</v>
+        <v>2017-06-08</v>
       </c>
       <c r="I4">
         <v>4200</v>
       </c>
       <c r="J4" t="str">
-        <v>today-28m</v>
+        <v>today+22m</v>
       </c>
       <c r="K4" t="str">
         <v>AquaTank Services</v>
@@ -4811,7 +5055,7 @@
         <v>operational</v>
       </c>
       <c r="M4" t="str">
-        <v>today-44d</v>
+        <v>today-55d</v>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -4840,16 +5084,16 @@
         <v>10m³</v>
       </c>
       <c r="G5" t="str">
-        <v>SID-959334</v>
+        <v>SID-759494</v>
       </c>
       <c r="H5" t="str">
-        <v>2017-02-19</v>
+        <v>2017-10-25</v>
       </c>
       <c r="I5">
         <v>3800</v>
       </c>
       <c r="J5" t="str">
-        <v>today-25m</v>
+        <v>today+4m</v>
       </c>
       <c r="K5" t="str">
         <v>AquaTank Services</v>
@@ -4858,7 +5102,7 @@
         <v>operational</v>
       </c>
       <c r="M5" t="str">
-        <v>today-65d</v>
+        <v>today-102d</v>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -4887,16 +5131,16 @@
         <v>Notifier</v>
       </c>
       <c r="G6" t="str">
-        <v>HON-691829</v>
+        <v>HON-184688</v>
       </c>
       <c r="H6" t="str">
-        <v>2022-09-13</v>
+        <v>2023-10-23</v>
       </c>
       <c r="I6">
         <v>9500</v>
       </c>
       <c r="J6" t="str">
-        <v>today+29m</v>
+        <v>today+23m</v>
       </c>
       <c r="K6" t="str">
         <v>FireSafe Lebanon</v>
@@ -4905,7 +5149,7 @@
         <v>operational</v>
       </c>
       <c r="M6" t="str">
-        <v>today-82d</v>
+        <v>today-84d</v>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -4934,16 +5178,16 @@
         <v>DS-7616</v>
       </c>
       <c r="G7" t="str">
-        <v>HIK-871507</v>
+        <v>HIK-246543</v>
       </c>
       <c r="H7" t="str">
-        <v>2020-09-19</v>
+        <v>2025-03-06</v>
       </c>
       <c r="I7">
         <v>3200</v>
       </c>
       <c r="J7" t="str">
-        <v>today-18m</v>
+        <v>today-39m</v>
       </c>
       <c r="K7" t="str">
         <v>SecureWatch</v>
@@ -4952,7 +5196,7 @@
         <v>operational</v>
       </c>
       <c r="M7" t="str">
-        <v>today-115d</v>
+        <v>today-94d</v>
       </c>
       <c r="N7" t="str">
         <v/>
@@ -4981,16 +5225,16 @@
         <v>Prisma</v>
       </c>
       <c r="G8" t="str">
-        <v>SCH-754588</v>
+        <v>SCH-502986</v>
       </c>
       <c r="H8" t="str">
-        <v>2017-02-04</v>
+        <v>2017-07-20</v>
       </c>
       <c r="I8">
         <v>6800</v>
       </c>
       <c r="J8" t="str">
-        <v>today+29m</v>
+        <v>today-24m</v>
       </c>
       <c r="K8" t="str">
         <v>Nakhle Electric</v>
@@ -4999,7 +5243,7 @@
         <v>operational</v>
       </c>
       <c r="M8" t="str">
-        <v>today-136d</v>
+        <v>today-111d</v>
       </c>
       <c r="N8" t="str">
         <v/>
@@ -5028,16 +5272,16 @@
         <v>BX-74</v>
       </c>
       <c r="G9" t="str">
-        <v>CAM-310880</v>
+        <v>CAM-761344</v>
       </c>
       <c r="H9" t="str">
-        <v>2017-03-15</v>
+        <v>2017-03-24</v>
       </c>
       <c r="I9">
         <v>2400</v>
       </c>
       <c r="J9" t="str">
-        <v>today+14m</v>
+        <v>today-33m</v>
       </c>
       <c r="K9" t="str">
         <v>SecureWatch</v>
@@ -5046,7 +5290,7 @@
         <v>operational</v>
       </c>
       <c r="M9" t="str">
-        <v>today-75d</v>
+        <v>today-92d</v>
       </c>
       <c r="N9" t="str">
         <v/>
@@ -5231,10 +5475,10 @@
         <v>3</v>
       </c>
       <c r="E2" t="str">
-        <v>today-12d</v>
+        <v>today-20d</v>
       </c>
       <c r="F2" t="str">
-        <v>today+78d</v>
+        <v>today+70d</v>
       </c>
       <c r="G2" t="str">
         <v>Schindler Lebanon</v>
@@ -5266,10 +5510,10 @@
         <v>12</v>
       </c>
       <c r="E3" t="str">
-        <v>today-235d</v>
+        <v>today-206d</v>
       </c>
       <c r="F3" t="str">
-        <v>today+125d</v>
+        <v>today+154d</v>
       </c>
       <c r="G3" t="str">
         <v>Schindler Lebanon</v>
@@ -5301,10 +5545,10 @@
         <v>6</v>
       </c>
       <c r="E4" t="str">
-        <v>today-52d</v>
+        <v>today-8d</v>
       </c>
       <c r="F4" t="str">
-        <v>today+128d</v>
+        <v>today+172d</v>
       </c>
       <c r="G4" t="str">
         <v>PowerGen Services</v>
@@ -5336,10 +5580,10 @@
         <v>6</v>
       </c>
       <c r="E5" t="str">
-        <v>today-95d</v>
+        <v>today-89d</v>
       </c>
       <c r="F5" t="str">
-        <v>today+85d</v>
+        <v>today+91d</v>
       </c>
       <c r="G5" t="str">
         <v>AquaTank Services</v>
@@ -5371,10 +5615,10 @@
         <v>6</v>
       </c>
       <c r="E6" t="str">
-        <v>today-162d</v>
+        <v>today-98d</v>
       </c>
       <c r="F6" t="str">
-        <v>today+18d</v>
+        <v>today+82d</v>
       </c>
       <c r="G6" t="str">
         <v>AquaTank Services</v>
@@ -5406,10 +5650,10 @@
         <v>12</v>
       </c>
       <c r="E7" t="str">
-        <v>today-317d</v>
+        <v>today-249d</v>
       </c>
       <c r="F7" t="str">
-        <v>today+43d</v>
+        <v>today+111d</v>
       </c>
       <c r="G7" t="str">
         <v>FireSafe Lebanon</v>
@@ -5441,10 +5685,10 @@
         <v>12</v>
       </c>
       <c r="E8" t="str">
-        <v>today-271d</v>
+        <v>today-212d</v>
       </c>
       <c r="F8" t="str">
-        <v>today+89d</v>
+        <v>today+148d</v>
       </c>
       <c r="G8" t="str">
         <v>SecureWatch</v>
@@ -5476,10 +5720,10 @@
         <v>12</v>
       </c>
       <c r="E9" t="str">
-        <v>today-174d</v>
+        <v>today-274d</v>
       </c>
       <c r="F9" t="str">
-        <v>today+186d</v>
+        <v>today+86d</v>
       </c>
       <c r="G9" t="str">
         <v>Nakhle Electric</v>
@@ -5511,10 +5755,10 @@
         <v>12</v>
       </c>
       <c r="E10" t="str">
-        <v>today-204d</v>
+        <v>today-237d</v>
       </c>
       <c r="F10" t="str">
-        <v>today+156d</v>
+        <v>today+123d</v>
       </c>
       <c r="G10" t="str">
         <v>SecureWatch</v>
@@ -5546,10 +5790,10 @@
         <v>3</v>
       </c>
       <c r="E11" t="str">
-        <v>today-79d</v>
+        <v>today-73d</v>
       </c>
       <c r="F11" t="str">
-        <v>today+17d</v>
+        <v>today+29d</v>
       </c>
       <c r="G11" t="str">
         <v>PestAway</v>

</xml_diff>